<commit_message>
Add new files and new features
</commit_message>
<xml_diff>
--- a/songs_questions.xlsx
+++ b/songs_questions.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D209"/>
+  <dimension ref="A1:D205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,7 +467,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="3">
@@ -478,16 +478,16 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Adele - Hello (Official Music Video)</t>
+          <t>24kGoldn - Mood (Official Video) ft. iann dior</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FAdele%20-%20Hello%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2F24kGoldn%20-%20Mood%20%28Official%20Video%29%20ft.%20iann%20dior.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="4">
@@ -498,16 +498,16 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Adele - Rolling in the Deep (Official Music Video)</t>
+          <t>Adele - Hello (Official Music Video)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FAdele%20-%20Rolling%20in%20the%20Deep%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FAdele%20-%20Hello%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="5">
@@ -518,16 +518,16 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Adele - Send My Love (To Your New Lover)</t>
+          <t>Adele - Rolling in the Deep (Official Music Video)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FAdele%20-%20Send%20My%20Love%20%28To%20Your%20New%20Lover%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FAdele%20-%20Rolling%20in%20the%20Deep%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="6">
@@ -538,16 +538,16 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Adele - Someone Like You (Official Music Video)</t>
+          <t>Adele - Send My Love (To Your New Lover)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FAdele%20-%20Someone%20Like%20You%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FAdele%20-%20Send%20My%20Love%20%28To%20Your%20New%20Lover%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="7">
@@ -558,16 +558,16 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Alan Walker &amp; Ava Max - Alone, Pt. II</t>
+          <t>Adele - Someone Like You (Official Music Video)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FAlan%20Walker%20%26%20Ava%20Max%20-%20Alone%2C%20Pt.%20II.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FAdele%20-%20Someone%20Like%20You%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="8">
@@ -578,16 +578,16 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Alan Walker - Alone</t>
+          <t>Alan Walker &amp; Ava Max - Alone, Pt. II</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FAlan%20Walker%20-%20Alone.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FAlan%20Walker%20%26%20Ava%20Max%20-%20Alone%2C%20Pt.%20II.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="9">
@@ -598,16 +598,16 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Alan Walker - Faded</t>
+          <t>Alan Walker - Alone</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FAlan%20Walker%20-%20Faded.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FAlan%20Walker%20-%20Alone.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="10">
@@ -618,16 +618,16 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Andy Grammer - Fresh Eyes (Official Music Video)</t>
+          <t>Alan Walker - Faded</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FAndy%20Grammer%20-%20Fresh%20Eyes%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FAlan%20Walker%20-%20Faded.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="11">
@@ -638,16 +638,16 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Anne-Marie &amp; James Arthur - Rewrite The Stars [from The Greatest Showman： Reimagined]</t>
+          <t>Andy Grammer - Fresh Eyes (Official Music Video)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FAnne-Marie%20%26%20James%20Arthur%20-%20Rewrite%20The%20Stars%20%5Bfrom%20The%20Greatest%20Showman%EF%BC%9A%20Reimagined%5D.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FAndy%20Grammer%20-%20Fresh%20Eyes%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="12">
@@ -658,16 +658,16 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Anne-Marie - 2002 [Official Video]</t>
+          <t>Anne-Marie &amp; James Arthur - Rewrite The Stars [from The Greatest Showman： Reimagined]</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FAnne-Marie%20-%202002%20%5BOfficial%20Video%5D.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FAnne-Marie%20%26%20James%20Arthur%20-%20Rewrite%20The%20Stars%20%5Bfrom%20The%20Greatest%20Showman%EF%BC%9A%20Reimagined%5D.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="13">
@@ -678,16 +678,16 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Arctic Monkeys - Do I Wanna Know？ (Official Video)</t>
+          <t>Anne-Marie - 2002 [Official Video]</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FArctic%20Monkeys%20-%20Do%20I%20Wanna%20Know%EF%BC%9F%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FAnne-Marie%20-%202002%20%5BOfficial%20Video%5D.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="14">
@@ -698,16 +698,16 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Ariana Grande - 7 rings (Official Video)</t>
+          <t>Arctic Monkeys - Do I Wanna Know？ (Official Video)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FAriana%20Grande%20-%207%20rings%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FArctic%20Monkeys%20-%20Do%20I%20Wanna%20Know%EF%BC%9F%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="15">
@@ -718,16 +718,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Ariana Grande - no tears left to cry (Official Video)</t>
+          <t>Ariana Grande - 7 rings (Official Video)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FAriana%20Grande%20-%20no%20tears%20left%20to%20cry%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FAriana%20Grande%20-%207%20rings%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="16">
@@ -738,16 +738,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Ariana Grande - thank u, next (Official Video)</t>
+          <t>Ariana Grande - no tears left to cry (Official Video)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FAriana%20Grande%20-%20thank%20u%2C%20next%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FAriana%20Grande%20-%20no%20tears%20left%20to%20cry%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="17">
@@ -758,16 +758,16 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Ariana Grande ft. Nicki Minaj - Side To Side (Official Video) ft. Nicki Minaj</t>
+          <t>Ariana Grande - thank u, next (Official Video)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FAriana%20Grande%20ft.%20Nicki%20Minaj%20-%20Side%20To%20Side%20%28Official%20Video%29%20ft.%20Nicki%20Minaj.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FAriana%20Grande%20-%20thank%20u%2C%20next%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="18">
@@ -778,16 +778,16 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>As We Learn(Play The Game)</t>
+          <t>Ariana Grande ft. Nicki Minaj - Side To Side (Official Video) ft. Nicki Minaj</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FAs%20We%20Learn%28Play%20The%20Game%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FAriana%20Grande%20ft.%20Nicki%20Minaj%20-%20Side%20To%20Side%20%28Official%20Video%29%20ft.%20Nicki%20Minaj.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="19">
@@ -798,16 +798,16 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Asia's Oldest Airport, Don Mueang in Bangkok ⧸ Vlog Review No. 344</t>
+          <t>As We Learn(Play The Game)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FAsia%27s%20Oldest%20Airport%2C%20Don%20Mueang%20in%20Bangkok%20%E2%A7%B8%20Vlog%20Review%20No.%20344.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FAs%20We%20Learn%28Play%20The%20Game%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="20">
@@ -827,7 +827,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="21">
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="22">
@@ -867,7 +867,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="23">
@@ -887,7 +887,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="24">
@@ -907,7 +907,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="25">
@@ -927,7 +927,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="26">
@@ -947,7 +947,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="27">
@@ -967,7 +967,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="28">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="29">
@@ -1007,7 +1007,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="30">
@@ -1027,7 +1027,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="31">
@@ -1047,7 +1047,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="32">
@@ -1067,7 +1067,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="33">
@@ -1087,7 +1087,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="34">
@@ -1107,7 +1107,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="35">
@@ -1127,7 +1127,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="36">
@@ -1147,7 +1147,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="37">
@@ -1167,7 +1167,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="38">
@@ -1187,7 +1187,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="39">
@@ -1207,7 +1207,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="40">
@@ -1227,7 +1227,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="41">
@@ -1247,7 +1247,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="42">
@@ -1267,7 +1267,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="43">
@@ -1287,7 +1287,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="44">
@@ -1307,7 +1307,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="45">
@@ -1327,7 +1327,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="46">
@@ -1347,7 +1347,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="47">
@@ -1367,7 +1367,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="48">
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="49">
@@ -1407,7 +1407,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="50">
@@ -1427,7 +1427,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="51">
@@ -1447,7 +1447,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="52">
@@ -1467,7 +1467,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="53">
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="54">
@@ -1498,16 +1498,16 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Daytime Walk at Tombori Riverwalk (Dotonbori Osaka) ⧸ Vlog Review No. 345</t>
+          <t>DJ Khaled - I'm The One ft. Justin Bieber, Quavo, Chance the Rapper, Lil Wayne</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FDaytime%20Walk%20at%20Tombori%20Riverwalk%20%28Dotonbori%20Osaka%29%20%E2%A7%B8%20Vlog%20Review%20No.%20345.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FDJ%20Khaled%20-%20I%27m%20The%20One%20ft.%20Justin%20Bieber%2C%20Quavo%2C%20Chance%20the%20Rapper%2C%20Lil%20Wayne.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="55">
@@ -1518,16 +1518,16 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>DJ Khaled - I'm The One ft. Justin Bieber, Quavo, Chance the Rapper, Lil Wayne</t>
+          <t>DJ Khaled - Wild Thoughts (Official Video) ft. Rihanna, Bryson Tiller</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FDJ%20Khaled%20-%20I%27m%20The%20One%20ft.%20Justin%20Bieber%2C%20Quavo%2C%20Chance%20the%20Rapper%2C%20Lil%20Wayne.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FDJ%20Khaled%20-%20Wild%20Thoughts%20%28Official%20Video%29%20ft.%20Rihanna%2C%20Bryson%20Tiller.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="56">
@@ -1538,16 +1538,16 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>DJ Khaled - Wild Thoughts (Official Video) ft. Rihanna, Bryson Tiller</t>
+          <t>DJ Snake - Let Me Love You ft. Justin Bieber</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FDJ%20Khaled%20-%20Wild%20Thoughts%20%28Official%20Video%29%20ft.%20Rihanna%2C%20Bryson%20Tiller.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FDJ%20Snake%20-%20Let%20Me%20Love%20You%20ft.%20Justin%20Bieber.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="57">
@@ -1558,16 +1558,16 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>DJ Snake - Let Me Love You ft. Justin Bieber</t>
+          <t>DJ Snake - Middle ft. Bipolar Sunshine</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FDJ%20Snake%20-%20Let%20Me%20Love%20You%20ft.%20Justin%20Bieber.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FDJ%20Snake%20-%20Middle%20ft.%20Bipolar%20Sunshine.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="58">
@@ -1578,16 +1578,16 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>DJ Snake - Middle ft. Bipolar Sunshine</t>
+          <t>DJ Snake - Taki Taki ft. Selena Gomez, Ozuna, Cardi B (Official Music Video)</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FDJ%20Snake%20-%20Middle%20ft.%20Bipolar%20Sunshine.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FDJ%20Snake%20-%20Taki%20Taki%20ft.%20Selena%20Gomez%2C%20Ozuna%2C%20Cardi%20B%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="59">
@@ -1598,16 +1598,16 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>DJ Snake - Taki Taki ft. Selena Gomez, Ozuna, Cardi B (Official Music Video)</t>
+          <t>DNCE - Cake By The Ocean</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FDJ%20Snake%20-%20Taki%20Taki%20ft.%20Selena%20Gomez%2C%20Ozuna%2C%20Cardi%20B%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FDNCE%20-%20Cake%20By%20The%20Ocean.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="60">
@@ -1618,16 +1618,16 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>DNCE - Cake By The Ocean</t>
+          <t>Drake - God's Plan</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FDNCE%20-%20Cake%20By%20The%20Ocean.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FDrake%20-%20God%27s%20Plan.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="61">
@@ -1638,16 +1638,16 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Drake - God's Plan</t>
+          <t>Drake - One Dance (Original)</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FDrake%20-%20God%27s%20Plan.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FDrake%20-%20One%20Dance%20%28Original%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="62">
@@ -1658,16 +1658,16 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Drake - One Dance (Original)</t>
+          <t>Dua Lipa - Don't Start Now (Official Music Video)</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FDrake%20-%20One%20Dance%20%28Original%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FDua%20Lipa%20-%20Don%27t%20Start%20Now%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="63">
@@ -1678,16 +1678,16 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Dua Lipa - Don't Start Now (Official Music Video)</t>
+          <t>Dua Lipa - IDGAF (Official Music Video)</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FDua%20Lipa%20-%20Don%27t%20Start%20Now%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FDua%20Lipa%20-%20IDGAF%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="64">
@@ -1698,16 +1698,16 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Dua Lipa - IDGAF (Official Music Video)</t>
+          <t>Dua Lipa - New Rules (Official Music Video)</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FDua%20Lipa%20-%20IDGAF%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FDua%20Lipa%20-%20New%20Rules%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="65">
@@ -1718,16 +1718,16 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Dua Lipa - New Rules (Official Music Video)</t>
+          <t>Ed Sheeran &amp; Justin Bieber - I Don't Care [Official Music Video]</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FDua%20Lipa%20-%20New%20Rules%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FEd%20Sheeran%20%26%20Justin%20Bieber%20-%20I%20Don%27t%20Care%20%5BOfficial%20Music%20Video%5D.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="66">
@@ -1738,16 +1738,16 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Ed Sheeran &amp; Justin Bieber - I Don't Care [Official Music Video]</t>
+          <t>Ed Sheeran - Castle On The Hill [Official Music Video]</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FEd%20Sheeran%20%26%20Justin%20Bieber%20-%20I%20Don%27t%20Care%20%5BOfficial%20Music%20Video%5D.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FEd%20Sheeran%20-%20Castle%20On%20The%20Hill%20%5BOfficial%20Music%20Video%5D.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="67">
@@ -1758,16 +1758,16 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Ed Sheeran - Castle On The Hill [Official Music Video]</t>
+          <t>Ed Sheeran - Perfect (Official Music Video)</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FEd%20Sheeran%20-%20Castle%20On%20The%20Hill%20%5BOfficial%20Music%20Video%5D.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FEd%20Sheeran%20-%20Perfect%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="68">
@@ -1778,16 +1778,16 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Ed Sheeran - Perfect (Official Music Video)</t>
+          <t>Ed Sheeran - Photograph (Official Music Video)</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FEd%20Sheeran%20-%20Perfect%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FEd%20Sheeran%20-%20Photograph%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="69">
@@ -1798,16 +1798,16 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Ed Sheeran - Photograph (Official Music Video)</t>
+          <t>Ed Sheeran - Shape of You (Official Music Video)</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FEd%20Sheeran%20-%20Photograph%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FEd%20Sheeran%20-%20Shape%20of%20You%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="70">
@@ -1818,16 +1818,16 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Ed Sheeran - Shape of You (Official Music Video)</t>
+          <t>Ed Sheeran - Thinking Out Loud (Official Music Video)</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FEd%20Sheeran%20-%20Shape%20of%20You%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FEd%20Sheeran%20-%20Thinking%20Out%20Loud%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="71">
@@ -1838,16 +1838,16 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Ed Sheeran - Thinking Out Loud (Official Music Video)</t>
+          <t>Ella Mai - Boo'd Up</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FEd%20Sheeran%20-%20Thinking%20Out%20Loud%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FElla%20Mai%20-%20Boo%27d%20Up.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="72">
@@ -1858,16 +1858,16 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Ella Mai - Boo'd Up</t>
+          <t>Ellie Goulding - Love Me Like You Do (Official Video)</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FElla%20Mai%20-%20Boo%27d%20Up.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FEllie%20Goulding%20-%20Love%20Me%20Like%20You%20Do%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="73">
@@ -1878,16 +1878,16 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Ellie Goulding - Love Me Like You Do (Official Video)</t>
+          <t>Field of Pain</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FEllie%20Goulding%20-%20Love%20Me%20Like%20You%20Do%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FField%20of%20Pain.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="74">
@@ -1898,16 +1898,16 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Field of Pain</t>
+          <t>Fifth Harmony - Worth It (Official Video) ft. Kid Ink</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FField%20of%20Pain.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FFifth%20Harmony%20-%20Worth%20It%20%28Official%20Video%29%20ft.%20Kid%20Ink.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="75">
@@ -1918,16 +1918,16 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Fifth Harmony - Worth It (Official Video) ft. Kid Ink</t>
+          <t>Finish My Plan - Don't Quit!</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FFifth%20Harmony%20-%20Worth%20It%20%28Official%20Video%29%20ft.%20Kid%20Ink.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FFinish%20My%20Plan%20-%20Don%27t%20Quit%21.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="76">
@@ -1938,16 +1938,16 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Finish My Plan - Don't Quit!</t>
+          <t>Fun.： We Are Young ft. Janelle Monáe [OFFICIAL VIDEO]</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FFinish%20My%20Plan%20-%20Don%27t%20Quit%21.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FFun.%EF%BC%9A%20We%20Are%20Young%20ft.%20Janelle%20Mon%C3%A1e%20%5BOFFICIAL%20VIDEO%5D.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="77">
@@ -1958,16 +1958,16 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Fun.： We Are Young ft. Janelle Monáe [OFFICIAL VIDEO]</t>
+          <t>Gawn Globel - Quien Eres Too ？</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FFun.%EF%BC%9A%20We%20Are%20Young%20ft.%20Janelle%20Mon%C3%A1e%20%5BOFFICIAL%20VIDEO%5D.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FGawn%20Globel%20-%20Quien%20Eres%20Too%20%EF%BC%9F.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="78">
@@ -1978,16 +1978,16 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Gawn Globel - Quien Eres Too ？</t>
+          <t>Gotye - Somebody That I Used To Know (feat. Kimbra) [Official Music Video]</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FGawn%20Globel%20-%20Quien%20Eres%20Too%20%EF%BC%9F.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FGotye%20-%20Somebody%20That%20I%20Used%20To%20Know%20%28feat.%20Kimbra%29%20%5BOfficial%20Music%20Video%5D.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="79">
@@ -1998,16 +1998,16 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Gotye - Somebody That I Used To Know (feat. Kimbra) [Official Music Video]</t>
+          <t>Halsey - Without Me</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FGotye%20-%20Somebody%20That%20I%20Used%20To%20Know%20%28feat.%20Kimbra%29%20%5BOfficial%20Music%20Video%5D.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FHalsey%20-%20Without%20Me.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="80">
@@ -2018,16 +2018,16 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Gransnow Okuibuki, Ski Resort Near Kyoto &amp; Osaka ⧸ Vlog Review No. 346</t>
+          <t>Harry Styles - Sign of the Times (Official Video)</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FGransnow%20Okuibuki%2C%20Ski%20Resort%20Near%20Kyoto%20%26%20Osaka%20%E2%A7%B8%20Vlog%20Review%20No.%20346.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FHarry%20Styles%20-%20Sign%20of%20the%20Times%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="81">
@@ -2038,16 +2038,16 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Halsey - Without Me</t>
+          <t>Iggy Azalea - Fancy ft. Charli XCX</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FHalsey%20-%20Without%20Me.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FIggy%20Azalea%20-%20Fancy%20ft.%20Charli%20XCX.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="82">
@@ -2058,16 +2058,16 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Harry Styles - Sign of the Times (Official Video)</t>
+          <t>Imagine Dragons - Believer (Official Music Video)</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FHarry%20Styles%20-%20Sign%20of%20the%20Times%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FImagine%20Dragons%20-%20Believer%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="83">
@@ -2078,16 +2078,16 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>IconSiam, Iconic Mall in Thailand ⧸ Vlog Review No. 341</t>
+          <t>Imagine Dragons - Radioactive</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FIconSiam%2C%20Iconic%20Mall%20in%20Thailand%20%E2%A7%B8%20Vlog%20Review%20No.%20341.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FImagine%20Dragons%20-%20Radioactive.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="84">
@@ -2098,16 +2098,16 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Iggy Azalea - Fancy ft. Charli XCX</t>
+          <t>Imagine Dragons - Thunder</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FIggy%20Azalea%20-%20Fancy%20ft.%20Charli%20XCX.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FImagine%20Dragons%20-%20Thunder.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="85">
@@ -2118,16 +2118,16 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Imagine Dragons - Believer (Official Music Video)</t>
+          <t>J Balvin, Willy William - Mi Gente (Official Video)</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FImagine%20Dragons%20-%20Believer%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FJ%20Balvin%2C%20Willy%20William%20-%20Mi%20Gente%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="86">
@@ -2138,16 +2138,16 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Imagine Dragons - Radioactive</t>
+          <t>James Arthur - Say You Won't Let Go</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FImagine%20Dragons%20-%20Radioactive.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FJames%20Arthur%20-%20Say%20You%20Won%27t%20Let%20Go.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="87">
@@ -2158,16 +2158,16 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Imagine Dragons - Thunder</t>
+          <t>Jason Derulo - Swalla (feat. Nicki Minaj &amp; Ty Dolla $ign) [Official Music Video]</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FImagine%20Dragons%20-%20Thunder.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FJason%20Derulo%20-%20Swalla%20%28feat.%20Nicki%20Minaj%20%26%20Ty%20Dolla%20%24ign%29%20%5BOfficial%20Music%20Video%5D.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="88">
@@ -2178,16 +2178,16 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>J Balvin, Willy William - Mi Gente (Official Video)</t>
+          <t>Jason Derulo - Wiggle feat. Snoop Dogg [Official Music Video]</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FJ%20Balvin%2C%20Willy%20William%20-%20Mi%20Gente%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FJason%20Derulo%20-%20Wiggle%20feat.%20Snoop%20Dogg%20%5BOfficial%20Music%20Video%5D.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="89">
@@ -2198,16 +2198,16 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>James Arthur - Say You Won't Let Go</t>
+          <t>Jason Derulo - ＂Want To Want Me＂ (Official Video)</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FJames%20Arthur%20-%20Say%20You%20Won%27t%20Let%20Go.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FJason%20Derulo%20-%20%EF%BC%82Want%20To%20Want%20Me%EF%BC%82%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="90">
@@ -2218,16 +2218,16 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Jason Derulo - Swalla (feat. Nicki Minaj &amp; Ty Dolla $ign) [Official Music Video]</t>
+          <t>Jessie J - Bang Bang ft. Ariana Grande, Nicki Minaj</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FJason%20Derulo%20-%20Swalla%20%28feat.%20Nicki%20Minaj%20%26%20Ty%20Dolla%20%24ign%29%20%5BOfficial%20Music%20Video%5D.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FJessie%20J%20-%20Bang%20Bang%20ft.%20Ariana%20Grande%2C%20Nicki%20Minaj.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="91">
@@ -2238,16 +2238,16 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Jason Derulo - Wiggle feat. Snoop Dogg [Official Music Video]</t>
+          <t>Jessie J - Domino (Official Video)</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FJason%20Derulo%20-%20Wiggle%20feat.%20Snoop%20Dogg%20%5BOfficial%20Music%20Video%5D.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FJessie%20J%20-%20Domino%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="92">
@@ -2258,16 +2258,16 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Jason Derulo - ＂Want To Want Me＂ (Official Video)</t>
+          <t>John Legend - All of Me (Official Video)</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FJason%20Derulo%20-%20%EF%BC%82Want%20To%20Want%20Me%EF%BC%82%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FJohn%20Legend%20-%20All%20of%20Me%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="93">
@@ -2278,16 +2278,16 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Jessie J - Bang Bang ft. Ariana Grande, Nicki Minaj</t>
+          <t>Jonas Brothers - Sucker (Official Video)</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FJessie%20J%20-%20Bang%20Bang%20ft.%20Ariana%20Grande%2C%20Nicki%20Minaj.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FJonas%20Brothers%20-%20Sucker%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="94">
@@ -2298,16 +2298,16 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Jessie J - Domino (Official Video)</t>
+          <t>Juice WRLD - Lucid Dreams (Official Music Video)</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FJessie%20J%20-%20Domino%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FJuice%20WRLD%20-%20Lucid%20Dreams%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="95">
@@ -2318,16 +2318,16 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>John Legend - All of Me (Official Video)</t>
+          <t>Justin Bieber - Beauty And A Beat (Official Music Video) ft. Nicki Minaj</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FJohn%20Legend%20-%20All%20of%20Me%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FJustin%20Bieber%20-%20Beauty%20And%20A%20Beat%20%28Official%20Music%20Video%29%20ft.%20Nicki%20Minaj.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="96">
@@ -2338,16 +2338,16 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Jonas Brothers - Sucker (Official Video)</t>
+          <t>Justin Bieber - Love Yourself (PURPOSE ： The Movement)</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FJonas%20Brothers%20-%20Sucker%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FJustin%20Bieber%20-%20Love%20Yourself%20%28PURPOSE%20%EF%BC%9A%20The%20Movement%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="97">
@@ -2358,16 +2358,16 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Juice WRLD - Lucid Dreams (Official Music Video)</t>
+          <t>Justin Bieber - Sorry (PURPOSE ： The Movement)</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FJuice%20WRLD%20-%20Lucid%20Dreams%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FJustin%20Bieber%20-%20Sorry%20%28PURPOSE%20%EF%BC%9A%20The%20Movement%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="98">
@@ -2378,16 +2378,16 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Justin Bieber - Beauty And A Beat (Official Music Video) ft. Nicki Minaj</t>
+          <t>Justin Timberlake - CAN'T STOP THE FEELING! (from DreamWorks Animation's ＂TROLLS＂) (Official Video)</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FJustin%20Bieber%20-%20Beauty%20And%20A%20Beat%20%28Official%20Music%20Video%29%20ft.%20Nicki%20Minaj.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FJustin%20Timberlake%20-%20CAN%27T%20STOP%20THE%20FEELING%21%20%28from%20DreamWorks%20Animation%27s%20%EF%BC%82TROLLS%EF%BC%82%29%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="99">
@@ -2398,16 +2398,16 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Justin Bieber - Love Yourself (PURPOSE ： The Movement)</t>
+          <t>Katy Perry - Bon Appétit (Official) ft. Migos</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FJustin%20Bieber%20-%20Love%20Yourself%20%28PURPOSE%20%EF%BC%9A%20The%20Movement%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FKaty%20Perry%20-%20Bon%20App%C3%A9tit%20%28Official%29%20ft.%20Migos.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="100">
@@ -2418,16 +2418,16 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Justin Bieber - Sorry (PURPOSE ： The Movement)</t>
+          <t>Katy Perry - Dark Horse ft. Juicy J</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FJustin%20Bieber%20-%20Sorry%20%28PURPOSE%20%EF%BC%9A%20The%20Movement%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FKaty%20Perry%20-%20Dark%20Horse%20ft.%20Juicy%20J.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="101">
@@ -2438,16 +2438,16 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Justin Timberlake - CAN'T STOP THE FEELING! (from DreamWorks Animation's ＂TROLLS＂) (Official Video)</t>
+          <t>Katy Perry - Firework (Official Music Video)</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FJustin%20Timberlake%20-%20CAN%27T%20STOP%20THE%20FEELING%21%20%28from%20DreamWorks%20Animation%27s%20%EF%BC%82TROLLS%EF%BC%82%29%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FKaty%20Perry%20-%20Firework%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="102">
@@ -2458,16 +2458,16 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Katy Perry - Bon Appétit (Official) ft. Migos</t>
+          <t>Katy Perry - Never Really Over (Official Video)</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FKaty%20Perry%20-%20Bon%20App%C3%A9tit%20%28Official%29%20ft.%20Migos.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FKaty%20Perry%20-%20Never%20Really%20Over%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="103">
@@ -2478,16 +2478,16 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Katy Perry - Dark Horse ft. Juicy J</t>
+          <t>Katy Perry - Roar</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FKaty%20Perry%20-%20Dark%20Horse%20ft.%20Juicy%20J.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FKaty%20Perry%20-%20Roar.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="104">
@@ -2498,16 +2498,16 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Katy Perry - Firework (Official Music Video)</t>
+          <t>Khalid &amp; Normani - Love Lies (Official Video)</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FKaty%20Perry%20-%20Firework%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FKhalid%20%26%20Normani%20-%20Love%20Lies%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="105">
@@ -2518,16 +2518,16 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Katy Perry - Never Really Over (Official Video)</t>
+          <t>Khalid - Better (Official Video)</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FKaty%20Perry%20-%20Never%20Really%20Over%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FKhalid%20-%20Better%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="106">
@@ -2538,16 +2538,16 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Katy Perry - Roar</t>
+          <t>Khalid - Talk (Official Video)</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FKaty%20Perry%20-%20Roar.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FKhalid%20-%20Talk%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="107">
@@ -2558,16 +2558,16 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Khalid &amp; Normani - Love Lies (Official Video)</t>
+          <t>Kygo, Selena Gomez - It Ain't Me (Official Video)</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FKhalid%20%26%20Normani%20-%20Love%20Lies%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FKygo%2C%20Selena%20Gomez%20-%20It%20Ain%27t%20Me%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="108">
@@ -2578,16 +2578,16 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Khalid - Better (Official Video)</t>
+          <t>Lady Gaga, Bradley Cooper - Shallow (from A Star Is Born) (Official Music Video)</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FKhalid%20-%20Better%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FLady%20Gaga%2C%20Bradley%20Cooper%20-%20Shallow%20%28from%20A%20Star%20Is%20Born%29%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="109">
@@ -2598,16 +2598,16 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Khalid - Talk (Official Video)</t>
+          <t>Lauv - I Like Me Better [Official Video]</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FKhalid%20-%20Talk%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FLauv%20-%20I%20Like%20Me%20Better%20%5BOfficial%20Video%5D.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="110">
@@ -2618,16 +2618,16 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Kygo, Selena Gomez - It Ain't Me (Official Video)</t>
+          <t>Lewis Capaldi - Someone You Loved</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FKygo%2C%20Selena%20Gomez%20-%20It%20Ain%27t%20Me%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FLewis%20Capaldi%20-%20Someone%20You%20Loved.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="111">
@@ -2638,16 +2638,16 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Lady Gaga, Bradley Cooper - Shallow (from A Star Is Born) (Official Music Video)</t>
+          <t>Liam Payne - Strip That Down ft. Quavo</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FLady%20Gaga%2C%20Bradley%20Cooper%20-%20Shallow%20%28from%20A%20Star%20Is%20Born%29%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FLiam%20Payne%20-%20Strip%20That%20Down%20ft.%20Quavo.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="112">
@@ -2658,16 +2658,16 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Lauv - I Like Me Better [Official Video]</t>
+          <t>Lil Nas X - Old Town Road (Official Video) ft. Billy Ray Cyrus</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FLauv%20-%20I%20Like%20Me%20Better%20%5BOfficial%20Video%5D.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FLil%20Nas%20X%20-%20Old%20Town%20Road%20%28Official%20Video%29%20ft.%20Billy%20Ray%20Cyrus.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="113">
@@ -2678,16 +2678,16 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Lewis Capaldi - Someone You Loved</t>
+          <t>Little Mix - Black Magic (Official Video)</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FLewis%20Capaldi%20-%20Someone%20You%20Loved.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FLittle%20Mix%20-%20Black%20Magic%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="114">
@@ -2698,16 +2698,16 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Liam Payne - Strip That Down ft. Quavo</t>
+          <t>Lizzo - Truth Hurts (Official Video)</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FLiam%20Payne%20-%20Strip%20That%20Down%20ft.%20Quavo.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FLizzo%20-%20Truth%20Hurts%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="115">
@@ -2718,16 +2718,16 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Lil Nas X - Old Town Road (Official Video) ft. Billy Ray Cyrus</t>
+          <t>Lorde - Royals (US Version)</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FLil%20Nas%20X%20-%20Old%20Town%20Road%20%28Official%20Video%29%20ft.%20Billy%20Ray%20Cyrus.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FLorde%20-%20Royals%20%28US%20Version%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="116">
@@ -2738,16 +2738,16 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Little Mix - Black Magic (Official Video)</t>
+          <t>Luis Fonsi, Daddy Yankee - Despacito (Audio) ft. Justin Bieber</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FLittle%20Mix%20-%20Black%20Magic%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FLuis%20Fonsi%2C%20Daddy%20Yankee%20-%20Despacito%20%28Audio%29%20ft.%20Justin%20Bieber.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="117">
@@ -2758,16 +2758,16 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Lizzo - Truth Hurts (Official Video)</t>
+          <t>Lukas Graham - 7 Years [Official Music Video]</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FLizzo%20-%20Truth%20Hurts%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FLukas%20Graham%20-%207%20Years%20%5BOfficial%20Music%20Video%5D.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="118">
@@ -2778,16 +2778,16 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Lorde - Royals (US Version)</t>
+          <t>MACKLEMORE &amp; RYAN LEWIS - CAN'T HOLD US FEAT. RAY DALTON (OFFICIAL MUSIC VIDEO)</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FLorde%20-%20Royals%20%28US%20Version%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMACKLEMORE%20%26%20RYAN%20LEWIS%20-%20CAN%27T%20HOLD%20US%20FEAT.%20RAY%20DALTON%20%28OFFICIAL%20MUSIC%20VIDEO%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="119">
@@ -2798,16 +2798,16 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Luis Fonsi, Daddy Yankee - Despacito (Audio) ft. Justin Bieber</t>
+          <t>MACKLEMORE &amp; RYAN LEWIS - THRIFT SHOP FEAT. WANZ (OFFICIAL VIDEO)</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FLuis%20Fonsi%2C%20Daddy%20Yankee%20-%20Despacito%20%28Audio%29%20ft.%20Justin%20Bieber.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMACKLEMORE%20%26%20RYAN%20LEWIS%20-%20THRIFT%20SHOP%20FEAT.%20WANZ%20%28OFFICIAL%20VIDEO%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="120">
@@ -2818,16 +2818,16 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Lukas Graham - 7 Years [Official Music Video]</t>
+          <t>MAGIC! - Rude (Official Video)</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FLukas%20Graham%20-%207%20Years%20%5BOfficial%20Music%20Video%5D.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMAGIC%21%20-%20Rude%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="121">
@@ -2838,16 +2838,16 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>MACKLEMORE &amp; RYAN LEWIS - CAN'T HOLD US FEAT. RAY DALTON (OFFICIAL MUSIC VIDEO)</t>
+          <t>Major Lazer &amp; DJ Snake - Lean On (feat. MØ) [Official 4K Music Video]</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMACKLEMORE%20%26%20RYAN%20LEWIS%20-%20CAN%27T%20HOLD%20US%20FEAT.%20RAY%20DALTON%20%28OFFICIAL%20MUSIC%20VIDEO%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMajor%20Lazer%20%26%20DJ%20Snake%20-%20Lean%20On%20%28feat.%20M%C3%98%29%20%5BOfficial%204K%20Music%20Video%5D.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="122">
@@ -2858,16 +2858,16 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>MACKLEMORE &amp; RYAN LEWIS - THRIFT SHOP FEAT. WANZ (OFFICIAL VIDEO)</t>
+          <t>Major Lazer - Cold Water (feat. Justin Bieber &amp; MØ) [Official Dance Video]</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMACKLEMORE%20%26%20RYAN%20LEWIS%20-%20THRIFT%20SHOP%20FEAT.%20WANZ%20%28OFFICIAL%20VIDEO%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMajor%20Lazer%20-%20Cold%20Water%20%28feat.%20Justin%20Bieber%20%26%20M%C3%98%29%20%5BOfficial%20Dance%20Video%5D.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="123">
@@ -2878,16 +2878,16 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>MAGIC! - Rude (Official Video)</t>
+          <t>Mariah Carey - Up Out My Face (Official Music Video) ft. Nicki Minaj</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMAGIC%21%20-%20Rude%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMariah%20Carey%20-%20Up%20Out%20My%20Face%20%28Official%20Music%20Video%29%20ft.%20Nicki%20Minaj.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="124">
@@ -2898,16 +2898,16 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Major Lazer &amp; DJ Snake - Lean On (feat. MØ) [Official 4K Music Video]</t>
+          <t>Mark Ronson - Uptown Funk (Official Video) ft. Bruno Mars</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMajor%20Lazer%20%26%20DJ%20Snake%20-%20Lean%20On%20%28feat.%20M%C3%98%29%20%5BOfficial%204K%20Music%20Video%5D.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMark%20Ronson%20-%20Uptown%20Funk%20%28Official%20Video%29%20ft.%20Bruno%20Mars.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="125">
@@ -2918,16 +2918,16 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Major Lazer - Cold Water (feat. Justin Bieber &amp; MØ) [Official Dance Video]</t>
+          <t>Maroon 5 - Don't Wanna Know (Official Music Video)</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMajor%20Lazer%20-%20Cold%20Water%20%28feat.%20Justin%20Bieber%20%26%20M%C3%98%29%20%5BOfficial%20Dance%20Video%5D.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMaroon%205%20-%20Don%27t%20Wanna%20Know%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="126">
@@ -2938,16 +2938,16 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Mariah Carey - Up Out My Face (Official Music Video) ft. Nicki Minaj</t>
+          <t>Maroon 5 - Girls Like You ft. Cardi B (Official Music Video)</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMariah%20Carey%20-%20Up%20Out%20My%20Face%20%28Official%20Music%20Video%29%20ft.%20Nicki%20Minaj.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMaroon%205%20-%20Girls%20Like%20You%20ft.%20Cardi%20B%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="127">
@@ -2958,16 +2958,16 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Mark Ronson - Uptown Funk (Official Video) ft. Bruno Mars</t>
+          <t>Maroon 5 - Memories (Official Video)</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMark%20Ronson%20-%20Uptown%20Funk%20%28Official%20Video%29%20ft.%20Bruno%20Mars.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMaroon%205%20-%20Memories%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="128">
@@ -2978,16 +2978,16 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Maroon 5 - Don't Wanna Know (Official Music Video)</t>
+          <t>Maroon 5 - Moves Like Jagger ft. Christina Aguilera (Official Music Video) ft. Christina Aguilera</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMaroon%205%20-%20Don%27t%20Wanna%20Know%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMaroon%205%20-%20Moves%20Like%20Jagger%20ft.%20Christina%20Aguilera%20%28Official%20Music%20Video%29%20ft.%20Christina%20Aguilera.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="129">
@@ -2998,16 +2998,16 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Maroon 5 - Girls Like You ft. Cardi B (Official Music Video)</t>
+          <t>Maroon 5 - Sugar (Official Music Video)</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMaroon%205%20-%20Girls%20Like%20You%20ft.%20Cardi%20B%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMaroon%205%20-%20Sugar%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="130">
@@ -3018,16 +3018,16 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Maroon 5 - Memories (Official Video)</t>
+          <t>Marshmello &amp; Anne-Marie - FRIENDS (Music Video) ＊OFFICIAL FRIENDZONE ANTHEM＊</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMaroon%205%20-%20Memories%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMarshmello%20%26%20Anne-Marie%20-%20FRIENDS%20%28Music%20Video%29%20%EF%BC%8AOFFICIAL%20FRIENDZONE%20ANTHEM%EF%BC%8A.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="131">
@@ -3038,16 +3038,16 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Maroon 5 - Moves Like Jagger ft. Christina Aguilera (Official Music Video) ft. Christina Aguilera</t>
+          <t>Marshmello - Alone (Official Music Video)</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMaroon%205%20-%20Moves%20Like%20Jagger%20ft.%20Christina%20Aguilera%20%28Official%20Music%20Video%29%20ft.%20Christina%20Aguilera.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMarshmello%20-%20Alone%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="132">
@@ -3058,16 +3058,16 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Maroon 5 - Sugar (Official Music Video)</t>
+          <t>Marshmello ft. Bastille - Happier (Official Music Video)</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMaroon%205%20-%20Sugar%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMarshmello%20ft.%20Bastille%20-%20Happier%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="133">
@@ -3078,16 +3078,16 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Marshmello &amp; Anne-Marie - FRIENDS (Music Video) ＊OFFICIAL FRIENDZONE ANTHEM＊</t>
+          <t>Meghan Trainor - All About That Bass (Official Video)</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMarshmello%20%26%20Anne-Marie%20-%20FRIENDS%20%28Music%20Video%29%20%EF%BC%8AOFFICIAL%20FRIENDZONE%20ANTHEM%EF%BC%8A.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMeghan%20Trainor%20-%20All%20About%20That%20Bass%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="134">
@@ -3098,16 +3098,16 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Marshmello - Alone (Official Music Video)</t>
+          <t>Meghan Trainor - Like I'm Gonna Lose You (Official Video) ft. John Legend</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMarshmello%20-%20Alone%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMeghan%20Trainor%20-%20Like%20I%27m%20Gonna%20Lose%20You%20%28Official%20Video%29%20ft.%20John%20Legend.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="135">
@@ -3118,16 +3118,16 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Marshmello ft. Bastille - Happier (Official Music Video)</t>
+          <t>Miley Cyrus - Wrecking Ball (Official Video)</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMarshmello%20ft.%20Bastille%20-%20Happier%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMiley%20Cyrus%20-%20Wrecking%20Ball%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="136">
@@ -3138,16 +3138,16 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Meghan Trainor - All About That Bass (Official Video)</t>
+          <t>Naughty Boy - La la la ft. Sam Smith (Official Video)</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMeghan%20Trainor%20-%20All%20About%20That%20Bass%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FNaughty%20Boy%20-%20La%20la%20la%20ft.%20Sam%20Smith%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="137">
@@ -3158,16 +3158,16 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Meghan Trainor - Like I'm Gonna Lose You (Official Video) ft. John Legend</t>
+          <t>Nicki Minaj - Super Bass (Official Video)</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMeghan%20Trainor%20-%20Like%20I%27m%20Gonna%20Lose%20You%20%28Official%20Video%29%20ft.%20John%20Legend.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FNicki%20Minaj%20-%20Super%20Bass%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="138">
@@ -3178,16 +3178,16 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Miley Cyrus - Wrecking Ball (Official Video)</t>
+          <t>One Direction - Best Song Ever</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FMiley%20Cyrus%20-%20Wrecking%20Ball%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FOne%20Direction%20-%20Best%20Song%20Ever.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="139">
@@ -3198,16 +3198,16 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Naughty Boy - La la la ft. Sam Smith (Official Video)</t>
+          <t>One Direction - Night Changes</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FNaughty%20Boy%20-%20La%20la%20la%20ft.%20Sam%20Smith%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FOne%20Direction%20-%20Night%20Changes.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="140">
@@ -3218,16 +3218,16 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Nicki Minaj - Super Bass (Official Video)</t>
+          <t>One Direction - One Thing</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FNicki%20Minaj%20-%20Super%20Bass%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FOne%20Direction%20-%20One%20Thing.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="141">
@@ -3238,16 +3238,16 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>One Direction - Best Song Ever</t>
+          <t>One Direction - What Makes You Beautiful (Official Video)</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FOne%20Direction%20-%20Best%20Song%20Ever.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FOne%20Direction%20-%20What%20Makes%20You%20Beautiful%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D141" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="142">
@@ -3258,16 +3258,16 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>One Direction - Night Changes</t>
+          <t>OneRepublic - Counting Stars</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FOne%20Direction%20-%20Night%20Changes.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FOneRepublic%20-%20Counting%20Stars.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="143">
@@ -3278,16 +3278,16 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>One Direction - One Thing</t>
+          <t>P!nk - Just Give Me A Reason ft. Nate Ruess</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FOne%20Direction%20-%20One%20Thing.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FP%21nk%20-%20Just%20Give%20Me%20A%20Reason%20ft.%20Nate%20Ruess.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="144">
@@ -3298,16 +3298,16 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>One Direction - What Makes You Beautiful (Official Video)</t>
+          <t>P!NK - What About Us (Official Video)</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FOne%20Direction%20-%20What%20Makes%20You%20Beautiful%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FP%21NK%20-%20What%20About%20Us%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="145">
@@ -3318,16 +3318,16 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>OneRepublic - Counting Stars</t>
+          <t>Panic! At The Disco - High Hopes (Official Video)</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FOneRepublic%20-%20Counting%20Stars.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FPanic%21%20At%20The%20Disco%20-%20High%20Hopes%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="146">
@@ -3338,16 +3338,16 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Our Recent Central World Bangkok Mall Tour ⧸ Vlog Review No. 343</t>
+          <t>Passenger ｜ Let Her Go (Official Video)</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FOur%20Recent%20Central%20World%20Bangkok%20Mall%20Tour%20%E2%A7%B8%20Vlog%20Review%20No.%20343.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FPassenger%20%EF%BD%9C%20Let%20Her%20Go%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="147">
@@ -3358,16 +3358,16 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>P!nk - Just Give Me A Reason ft. Nate Ruess</t>
+          <t>Pharrell Williams - Happy (Official Video)</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FP%21nk%20-%20Just%20Give%20Me%20A%20Reason%20ft.%20Nate%20Ruess.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FPharrell%20Williams%20-%20Happy%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="148">
@@ -3378,16 +3378,16 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>P!NK - What About Us (Official Video)</t>
+          <t>Post Malone - Better Now</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FP%21NK%20-%20What%20About%20Us%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FPost%20Malone%20-%20Better%20Now.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="149">
@@ -3398,16 +3398,16 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Panic! At The Disco - High Hopes (Official Video)</t>
+          <t>Post Malone - Circles</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FPanic%21%20At%20The%20Disco%20-%20High%20Hopes%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FPost%20Malone%20-%20Circles.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="150">
@@ -3418,16 +3418,16 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Passenger ｜ Let Her Go (Official Video)</t>
+          <t>Post Malone - Congratulations (Official Music Video) ft. Quavo</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FPassenger%20%EF%BD%9C%20Let%20Her%20Go%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FPost%20Malone%20-%20Congratulations%20%28Official%20Music%20Video%29%20ft.%20Quavo.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="151">
@@ -3438,16 +3438,16 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Pharrell Williams - Happy (Official Video)</t>
+          <t>Post Malone - Psycho (Official Music Video) ft. Ty Dolla $ign</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FPharrell%20Williams%20-%20Happy%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FPost%20Malone%20-%20Psycho%20%28Official%20Music%20Video%29%20ft.%20Ty%20Dolla%20%24ign.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="152">
@@ -3458,16 +3458,16 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Post Malone - Better Now</t>
+          <t>Post Malone - rockstar (Official Music Video) ft. 21 Savage</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FPost%20Malone%20-%20Better%20Now.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FPost%20Malone%20-%20rockstar%20%28Official%20Music%20Video%29%20ft.%2021%20Savage.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="153">
@@ -3478,16 +3478,16 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Post Malone - Circles</t>
+          <t>Post Malone, Swae Lee - Sunflower (Spider-Man： Into the Spider-Verse)</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FPost%20Malone%20-%20Circles.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FPost%20Malone%2C%20Swae%20Lee%20-%20Sunflower%20%28Spider-Man%EF%BC%9A%20Into%20the%20Spider-Verse%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="154">
@@ -3498,16 +3498,16 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Post Malone - Congratulations (Official Music Video) ft. Quavo</t>
+          <t>R. City - Locked Away (Official Video) ft. Adam Levine</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FPost%20Malone%20-%20Congratulations%20%28Official%20Music%20Video%29%20ft.%20Quavo.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FR.%20City%20-%20Locked%20Away%20%28Official%20Video%29%20ft.%20Adam%20Levine.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="155">
@@ -3518,16 +3518,16 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Post Malone - Psycho (Official Music Video) ft. Ty Dolla $ign</t>
+          <t>Rachel Platten - Fight Song (Official Video)</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FPost%20Malone%20-%20Psycho%20%28Official%20Music%20Video%29%20ft.%20Ty%20Dolla%20%24ign.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FRachel%20Platten%20-%20Fight%20Song%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="156">
@@ -3538,16 +3538,16 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Post Malone - rockstar (Official Music Video) ft. 21 Savage</t>
+          <t>Rihanna - We Found Love ft. Calvin Harris</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FPost%20Malone%20-%20rockstar%20%28Official%20Music%20Video%29%20ft.%2021%20Savage.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FRihanna%20-%20We%20Found%20Love%20ft.%20Calvin%20Harris.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="157">
@@ -3558,16 +3558,16 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Post Malone, Swae Lee - Sunflower (Spider-Man： Into the Spider-Verse)</t>
+          <t>Rihanna - Work (Explicit) ft. Drake</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FPost%20Malone%2C%20Swae%20Lee%20-%20Sunflower%20%28Spider-Man%EF%BC%9A%20Into%20the%20Spider-Verse%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FRihanna%20-%20Work%20%28Explicit%29%20ft.%20Drake.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D157" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="158">
@@ -3578,16 +3578,16 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>R. City - Locked Away (Official Video) ft. Adam Levine</t>
+          <t>ROMANI - RATED R (Official Video)</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FR.%20City%20-%20Locked%20Away%20%28Official%20Video%29%20ft.%20Adam%20Levine.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FROMANI%20-%20RATED%20R%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="159">
@@ -3598,16 +3598,16 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Rachel Platten - Fight Song (Official Video)</t>
+          <t>Rosa Linn - Snap - (Official Eurovision Music Video)</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FRachel%20Platten%20-%20Fight%20Song%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FRosa%20Linn%20-%20Snap%20-%20%28Official%20Eurovision%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="160">
@@ -3618,16 +3618,16 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Rihanna - We Found Love ft. Calvin Harris</t>
+          <t>Sam Smith - How Do You Sleep？ (Official Music Video)</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FRihanna%20-%20We%20Found%20Love%20ft.%20Calvin%20Harris.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FSam%20Smith%20-%20How%20Do%20You%20Sleep%EF%BC%9F%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="161">
@@ -3638,16 +3638,16 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Rihanna - Work (Explicit) ft. Drake</t>
+          <t>Sam Smith - I'm Not The Only One (Official Music Video)</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FRihanna%20-%20Work%20%28Explicit%29%20ft.%20Drake.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FSam%20Smith%20-%20I%27m%20Not%20The%20Only%20One%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="162">
@@ -3658,16 +3658,16 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>ROMANI - RATED R (Official Video)</t>
+          <t>Sam Smith - Stay With Me (Official Music Video)</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FROMANI%20-%20RATED%20R%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FSam%20Smith%20-%20Stay%20With%20Me%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="163">
@@ -3678,16 +3678,16 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Sam Smith - How Do You Sleep？ (Official Music Video)</t>
+          <t>Sam Smith - Too Good At Goodbyes</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FSam%20Smith%20-%20How%20Do%20You%20Sleep%EF%BC%9F%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FSam%20Smith%20-%20Too%20Good%20At%20Goodbyes.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="164">
@@ -3698,16 +3698,16 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Sam Smith - I'm Not The Only One (Official Music Video)</t>
+          <t>Sam Smith, Normani - Dancing With A Stranger (Official Music Video)</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FSam%20Smith%20-%20I%27m%20Not%20The%20Only%20One%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FSam%20Smith%2C%20Normani%20-%20Dancing%20With%20A%20Stranger%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="165">
@@ -3718,16 +3718,16 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Sam Smith - Stay With Me (Official Music Video)</t>
+          <t>Selena Gomez - Bad Liar</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FSam%20Smith%20-%20Stay%20With%20Me%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FSelena%20Gomez%20-%20Bad%20Liar.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D165" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="166">
@@ -3738,16 +3738,16 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Sam Smith - Too Good At Goodbyes</t>
+          <t>Selena Gomez - Come &amp; Get It</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FSam%20Smith%20-%20Too%20Good%20At%20Goodbyes.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FSelena%20Gomez%20-%20Come%20%26%20Get%20It.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="167">
@@ -3758,16 +3758,16 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Sam Smith, Normani - Dancing With A Stranger (Official Music Video)</t>
+          <t>Selena Gomez - Lose You To Love Me (Official Music Video)</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FSam%20Smith%2C%20Normani%20-%20Dancing%20With%20A%20Stranger%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FSelena%20Gomez%20-%20Lose%20You%20To%20Love%20Me%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="168">
@@ -3778,16 +3778,16 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>Selena Gomez - Bad Liar</t>
+          <t>Selena Gomez - Same Old Love</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FSelena%20Gomez%20-%20Bad%20Liar.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FSelena%20Gomez%20-%20Same%20Old%20Love.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="169">
@@ -3798,16 +3798,16 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Selena Gomez - Come &amp; Get It</t>
+          <t>Selena Gomez - The Heart Wants What It Wants (Official Video)</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FSelena%20Gomez%20-%20Come%20%26%20Get%20It.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FSelena%20Gomez%20-%20The%20Heart%20Wants%20What%20It%20Wants%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="170">
@@ -3818,16 +3818,16 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Selena Gomez - Lose You To Love Me (Official Music Video)</t>
+          <t>Selena Gomez, Marshmello - Wolves</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FSelena%20Gomez%20-%20Lose%20You%20To%20Love%20Me%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FSelena%20Gomez%2C%20Marshmello%20-%20Wolves.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="171">
@@ -3838,16 +3838,16 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Selena Gomez - Same Old Love</t>
+          <t>Shawn Mendes - If I Can't Have You (Official Music Video)</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FSelena%20Gomez%20-%20Same%20Old%20Love.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FShawn%20Mendes%20-%20If%20I%20Can%27t%20Have%20You%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="172">
@@ -3858,16 +3858,16 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Selena Gomez - The Heart Wants What It Wants (Official Video)</t>
+          <t>Shawn Mendes - In My Blood</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FSelena%20Gomez%20-%20The%20Heart%20Wants%20What%20It%20Wants%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FShawn%20Mendes%20-%20In%20My%20Blood.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="173">
@@ -3878,16 +3878,16 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Selena Gomez, Marshmello - Wolves</t>
+          <t>Shawn Mendes - Stitches (Official Music Video)</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FSelena%20Gomez%2C%20Marshmello%20-%20Wolves.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FShawn%20Mendes%20-%20Stitches%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="174">
@@ -3898,16 +3898,16 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Shawn Mendes - If I Can't Have You (Official Music Video)</t>
+          <t>Shawn Mendes - There's Nothing Holdin' Me Back (Official Music Video)</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FShawn%20Mendes%20-%20If%20I%20Can%27t%20Have%20You%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FShawn%20Mendes%20-%20There%27s%20Nothing%20Holdin%27%20Me%20Back%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="175">
@@ -3918,16 +3918,16 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Shawn Mendes - In My Blood</t>
+          <t>Shawn Mendes - Treat You Better</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FShawn%20Mendes%20-%20In%20My%20Blood.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FShawn%20Mendes%20-%20Treat%20You%20Better.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="176">
@@ -3938,16 +3938,16 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Shawn Mendes - Stitches (Official Music Video)</t>
+          <t>Shawn Mendes, Camila Cabello - Señorita</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FShawn%20Mendes%20-%20Stitches%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FShawn%20Mendes%2C%20Camila%20Cabello%20-%20Se%C3%B1orita.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="177">
@@ -3958,16 +3958,16 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Shawn Mendes - There's Nothing Holdin' Me Back (Official Music Video)</t>
+          <t>Sia - Chandelier (Official Video)</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FShawn%20Mendes%20-%20There%27s%20Nothing%20Holdin%27%20Me%20Back%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FSia%20-%20Chandelier%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D177" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="178">
@@ -3978,16 +3978,16 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Shawn Mendes - Treat You Better</t>
+          <t>Sia - Cheap Thrills (Official Lyric Video) ft. Sean Paul</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FShawn%20Mendes%20-%20Treat%20You%20Better.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FSia%20-%20Cheap%20Thrills%20%28Official%20Lyric%20Video%29%20ft.%20Sean%20Paul.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="179">
@@ -3998,16 +3998,16 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Shawn Mendes, Camila Cabello - Señorita</t>
+          <t>Snoop Dogg - Step ft. Swizz Beatz (Visualizer)</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FShawn%20Mendes%2C%20Camila%20Cabello%20-%20Se%C3%B1orita.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FSnoop%20Dogg%20-%20Step%20ft.%20Swizz%20Beatz%20%28Visualizer%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="180">
@@ -4018,16 +4018,16 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Sia - Chandelier (Official Video)</t>
+          <t>Snoop Dogg - Stop Counting My Poccets (Official Music Video)</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FSia%20-%20Chandelier%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FSnoop%20Dogg%20-%20Stop%20Counting%20My%20Poccets%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="181">
@@ -4038,16 +4038,16 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Sia - Cheap Thrills (Official Lyric Video) ft. Sean Paul</t>
+          <t>Sometimes - TackEm</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FSia%20-%20Cheap%20Thrills%20%28Official%20Lyric%20Video%29%20ft.%20Sean%20Paul.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FSometimes%20-%20TackEm.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="182">
@@ -4058,16 +4058,16 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Snoop Dogg - Step ft. Swizz Beatz (Visualizer)</t>
+          <t>Taylor Swift - Bad Blood ft. Kendrick Lamar</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FSnoop%20Dogg%20-%20Step%20ft.%20Swizz%20Beatz%20%28Visualizer%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FTaylor%20Swift%20-%20Bad%20Blood%20ft.%20Kendrick%20Lamar.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="183">
@@ -4078,16 +4078,16 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Snoop Dogg - Stop Counting My Poccets (Official Music Video)</t>
+          <t>Taylor Swift - Blank Space</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FSnoop%20Dogg%20-%20Stop%20Counting%20My%20Poccets%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FTaylor%20Swift%20-%20Blank%20Space.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="184">
@@ -4098,16 +4098,16 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Snow Play at Gransnow Okuibuki Near Kyoto &amp; Osaka ⧸ Vlog Review No. 347</t>
+          <t>Taylor Swift - Look What You Made Me Do</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FSnow%20Play%20at%20Gransnow%20Okuibuki%20Near%20Kyoto%20%26%20Osaka%20%E2%A7%B8%20Vlog%20Review%20No.%20347.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FTaylor%20Swift%20-%20Look%20What%20You%20Made%20Me%20Do.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="185">
@@ -4118,16 +4118,16 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Sometimes - TackEm</t>
+          <t>Taylor Swift - Shake It Off</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FSometimes%20-%20TackEm.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FTaylor%20Swift%20-%20Shake%20It%20Off.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="186">
@@ -4138,16 +4138,16 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Taylor Swift - Bad Blood ft. Kendrick Lamar</t>
+          <t>The Chainsmokers &amp; Coldplay - Something Just Like This (Official Lyric Video)</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FTaylor%20Swift%20-%20Bad%20Blood%20ft.%20Kendrick%20Lamar.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FThe%20Chainsmokers%20%26%20Coldplay%20-%20Something%20Just%20Like%20This%20%28Official%20Lyric%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="187">
@@ -4158,16 +4158,16 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Taylor Swift - Blank Space</t>
+          <t>The Chainsmokers - Closer (Lyric) ft. Halsey</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FTaylor%20Swift%20-%20Blank%20Space.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FThe%20Chainsmokers%20-%20Closer%20%28Lyric%29%20ft.%20Halsey.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="188">
@@ -4178,16 +4178,16 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Taylor Swift - Look What You Made Me Do</t>
+          <t>The Chainsmokers - Don't Let Me Down (Official Video) ft. Daya</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FTaylor%20Swift%20-%20Look%20What%20You%20Made%20Me%20Do.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FThe%20Chainsmokers%20-%20Don%27t%20Let%20Me%20Down%20%28Official%20Video%29%20ft.%20Daya.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="189">
@@ -4198,16 +4198,16 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Taylor Swift - Shake It Off</t>
+          <t>The Chainsmokers - Roses (Official Lyric Video) ft. ROZES</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FTaylor%20Swift%20-%20Shake%20It%20Off.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FThe%20Chainsmokers%20-%20Roses%20%28Official%20Lyric%20Video%29%20ft.%20ROZES.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="190">
@@ -4218,16 +4218,16 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>The Chainsmokers &amp; Coldplay - Something Just Like This (Official Lyric Video)</t>
+          <t>The Lumineers - Ho Hey (Official Video)</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FThe%20Chainsmokers%20%26%20Coldplay%20-%20Something%20Just%20Like%20This%20%28Official%20Lyric%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FThe%20Lumineers%20-%20Ho%20Hey%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="191">
@@ -4238,16 +4238,16 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>The Chainsmokers - Closer (Lyric) ft. Halsey</t>
+          <t>The Weeknd - Can't Feel My Face (Official Video)</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FThe%20Chainsmokers%20-%20Closer%20%28Lyric%29%20ft.%20Halsey.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FThe%20Weeknd%20-%20Can%27t%20Feel%20My%20Face%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="192">
@@ -4258,16 +4258,16 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>The Chainsmokers - Don't Let Me Down (Official Video) ft. Daya</t>
+          <t>The Weeknd - I Feel It Coming ft. Daft Punk (Official Video)</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FThe%20Chainsmokers%20-%20Don%27t%20Let%20Me%20Down%20%28Official%20Video%29%20ft.%20Daya.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FThe%20Weeknd%20-%20I%20Feel%20It%20Coming%20ft.%20Daft%20Punk%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="193">
@@ -4278,16 +4278,16 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>The Chainsmokers - Roses (Official Lyric Video) ft. ROZES</t>
+          <t>The Weeknd - Starboy ft. Daft Punk (Official Video) ft. Daft Punk</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FThe%20Chainsmokers%20-%20Roses%20%28Official%20Lyric%20Video%29%20ft.%20ROZES.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FThe%20Weeknd%20-%20Starboy%20ft.%20Daft%20Punk%20%28Official%20Video%29%20ft.%20Daft%20Punk.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="194">
@@ -4298,16 +4298,16 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>The Lumineers - Ho Hey (Official Video)</t>
+          <t>TONES AND I - DANCE MONKEY (OFFICIAL VIDEO)</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FThe%20Lumineers%20-%20Ho%20Hey%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FTONES%20AND%20I%20-%20DANCE%20MONKEY%20%28OFFICIAL%20VIDEO%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="195">
@@ -4318,16 +4318,16 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>The Weeknd - Can't Feel My Face (Official Video)</t>
+          <t>Travis Scott - SICKO MODE (Official Video) ft. Drake</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FThe%20Weeknd%20-%20Can%27t%20Feel%20My%20Face%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FTravis%20Scott%20-%20SICKO%20MODE%20%28Official%20Video%29%20ft.%20Drake.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D195" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="196">
@@ -4338,16 +4338,16 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>The Weeknd - I Feel It Coming ft. Daft Punk (Official Video)</t>
+          <t>twenty one pilots - Ride (Official Video)</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FThe%20Weeknd%20-%20I%20Feel%20It%20Coming%20ft.%20Daft%20Punk%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2Ftwenty%20one%20pilots%20-%20Ride%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="197">
@@ -4358,16 +4358,16 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>The Weeknd - Starboy ft. Daft Punk (Official Video) ft. Daft Punk</t>
+          <t>twenty one pilots： Heathens (from Suicide Squad： The Album) [OFFICIAL VIDEO]</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FThe%20Weeknd%20-%20Starboy%20ft.%20Daft%20Punk%20%28Official%20Video%29%20ft.%20Daft%20Punk.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2Ftwenty%20one%20pilots%EF%BC%9A%20Heathens%20%28from%20Suicide%20Squad%EF%BC%9A%20The%20Album%29%20%5BOFFICIAL%20VIDEO%5D.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="198">
@@ -4378,16 +4378,16 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>TONES AND I - DANCE MONKEY (OFFICIAL VIDEO)</t>
+          <t>twenty one pilots： Stressed Out [OFFICIAL VIDEO]</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FTONES%20AND%20I%20-%20DANCE%20MONKEY%20%28OFFICIAL%20VIDEO%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2Ftwenty%20one%20pilots%EF%BC%9A%20Stressed%20Out%20%5BOFFICIAL%20VIDEO%5D.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="199">
@@ -4398,16 +4398,16 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Travis Scott - SICKO MODE (Official Video) ft. Drake</t>
+          <t>WALK THE MOON - Shut Up and Dance (Official Video)</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FTravis%20Scott%20-%20SICKO%20MODE%20%28Official%20Video%29%20ft.%20Drake.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FWALK%20THE%20MOON%20-%20Shut%20Up%20and%20Dance%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D199" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="200">
@@ -4418,16 +4418,16 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>twenty one pilots - Ride (Official Video)</t>
+          <t>Wiz Khalifa - See You Again ft. Charlie Puth [Official Video] Furious 7 Soundtrack</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2Ftwenty%20one%20pilots%20-%20Ride%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FWiz%20Khalifa%20-%20See%20You%20Again%20ft.%20Charlie%20Puth%20%5BOfficial%20Video%5D%20Furious%207%20Soundtrack.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="201">
@@ -4438,16 +4438,16 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>twenty one pilots： Heathens (from Suicide Squad： The Album) [OFFICIAL VIDEO]</t>
+          <t>XXXTENTACION - SAD!</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2Ftwenty%20one%20pilots%EF%BC%9A%20Heathens%20%28from%20Suicide%20Squad%EF%BC%9A%20The%20Album%29%20%5BOFFICIAL%20VIDEO%5D.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FXXXTENTACION%20-%20SAD%21.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="202">
@@ -4458,16 +4458,16 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>twenty one pilots： Stressed Out [OFFICIAL VIDEO]</t>
+          <t>Y2K, bbno$ - Lalala (Official Video)</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2Ftwenty%20one%20pilots%EF%BC%9A%20Stressed%20Out%20%5BOFFICIAL%20VIDEO%5D.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FY2K%2C%20bbno%24%20-%20Lalala%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="203">
@@ -4478,16 +4478,16 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>WALK THE MOON - Shut Up and Dance (Official Video)</t>
+          <t>ZAYN - Dusk Till Dawn (Official Video) ft. Sia</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FWALK%20THE%20MOON%20-%20Shut%20Up%20and%20Dance%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FZAYN%20-%20Dusk%20Till%20Dawn%20%28Official%20Video%29%20ft.%20Sia.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="204">
@@ -4498,16 +4498,16 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>Wiz Khalifa - See You Again ft. Charlie Puth [Official Video] Furious 7 Soundtrack</t>
+          <t>Zedd, Alessia Cara - Stay (Official Music Video)</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FWiz%20Khalifa%20-%20See%20You%20Again%20ft.%20Charlie%20Puth%20%5BOfficial%20Video%5D%20Furious%207%20Soundtrack.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FZedd%2C%20Alessia%20Cara%20-%20Stay%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D204" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="205">
@@ -4518,96 +4518,16 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>XXXTENTACION - SAD!</t>
+          <t>Zedd, Maren Morris, Grey - The Middle (Official Music Video)</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FXXXTENTACION%20-%20SAD%21.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
+          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FZedd%2C%20Maren%20Morris%2C%20Grey%20-%20The%20Middle%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="206">
-      <c r="A206" t="inlineStr">
-        <is>
-          <t>ما اسم الأغنية؟</t>
-        </is>
-      </c>
-      <c r="B206" t="inlineStr">
-        <is>
-          <t>Y2K, bbno$ - Lalala (Official Video)</t>
-        </is>
-      </c>
-      <c r="C206" t="inlineStr">
-        <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FY2K%2C%20bbno%24%20-%20Lalala%20%28Official%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
-        </is>
-      </c>
-      <c r="D206" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="207">
-      <c r="A207" t="inlineStr">
-        <is>
-          <t>ما اسم الأغنية؟</t>
-        </is>
-      </c>
-      <c r="B207" t="inlineStr">
-        <is>
-          <t>ZAYN - Dusk Till Dawn (Official Video) ft. Sia</t>
-        </is>
-      </c>
-      <c r="C207" t="inlineStr">
-        <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FZAYN%20-%20Dusk%20Till%20Dawn%20%28Official%20Video%29%20ft.%20Sia.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
-        </is>
-      </c>
-      <c r="D207" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="208">
-      <c r="A208" t="inlineStr">
-        <is>
-          <t>ما اسم الأغنية؟</t>
-        </is>
-      </c>
-      <c r="B208" t="inlineStr">
-        <is>
-          <t>Zedd, Alessia Cara - Stay (Official Music Video)</t>
-        </is>
-      </c>
-      <c r="C208" t="inlineStr">
-        <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FZedd%2C%20Alessia%20Cara%20-%20Stay%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
-        </is>
-      </c>
-      <c r="D208" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="209">
-      <c r="A209" t="inlineStr">
-        <is>
-          <t>ما اسم الأغنية؟</t>
-        </is>
-      </c>
-      <c r="B209" t="inlineStr">
-        <is>
-          <t>Zedd, Maren Morris, Grey - The Middle (Official Music Video)</t>
-        </is>
-      </c>
-      <c r="C209" t="inlineStr">
-        <is>
-          <t>https://firebasestorage.googleapis.com/v0/b/henka-game.firebasestorage.app/o/songs%2FZedd%2C%20Maren%20Morris%2C%20Grey%20-%20The%20Middle%20%28Official%20Music%20Video%29.webm?alt=media&amp;token=649fe6e0-05b5-4639-acb2-022f90180412</t>
-        </is>
-      </c>
-      <c r="D209" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
   </sheetData>

</xml_diff>